<commit_message>
Atualiza para 4 provedores, n=3 (60 execucoes)
</commit_message>
<xml_diff>
--- a/dados/rubrica-tcc.xlsx
+++ b/dados/rubrica-tcc.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="148">
   <si>
     <t xml:space="preserve">Rubrica de avaliacao — TCC LLMs x Complexidade Progressiva</t>
   </si>
@@ -340,6 +340,108 @@
   </si>
   <si>
     <t xml:space="preserve">outputs/nivel-4-seguranca-autenticacao-e-autorizacao/gemini/tentativa-2.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">groq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">openai/gpt-oss-120b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado em teste local pelo autor (28/08/2026): duas execucoes consecutivas, users.csv com duas linhas, sem sobrescrever a anterior. Nao testavel no sandbox automatizado por exigir terminal real (prompt-sync) - mesma categoria do Gemini nivel 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Via argumento de linha de comando (nao interativo). Testado: duas execucoes, CSV com 2 linhas, sem sobrescrever.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRUD completo via commander (add/list/update/delete), com confirmacao y/n na remocao. Testado: cadastro, duplicidade de e-mail rejeitada, atualizacao, remocao - tudo funcional.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado em teste local pelo autor (28/08/2026), apos correcao de 2 dependencias (better-sqlite3 e inquirer, ver Seccao metodologica): cadastro, listagem e bloqueio de e-mail duplicado (mensagem amigavel, sem prosseguir) - tudo funcional. Nao testavel no sandbox automatizado por exigir terminal real (inquirer) - mesma categoria do Gemini nivel 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 correcao manual: package.json continha uma linha de comentario invalida ('// package.json') dentro do JSON, quebrando o parsing - removida. Apos a correcao: CRUD completo via /users, 409 correto para e-mail duplicado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 correcao manual: codigo importava o pacote 'sqlite' (wrapper de promises), mas so 'sqlite3' estava declarado no package.json - adicionado. CRUD funcional, mas retorna 400 (nao 409) para e-mail duplicado - inconsistente com a tentativa 1 do mesmo modelo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rotas em /api/users (nao /users, como a descricao inicial sugeria). Campo 'age' em vez de 'birthdate' - interpretacao valida, pois o nivel nao especifica campos. CRUD completo testado, 409 correto; DELETE retorna 200 em vez de 204 (estilo, nao erro).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRUD completo funcional, 409 correto, DELETE 204. Boas praticas com ressalva: um stack trace bruto do SQLite (constraint de e-mail duplicado) e impresso no console do servidor mesmo a API respondendo corretamente ao cliente - vazamento de log, nao de seguranca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 correcoes manuais: dependencia 'dotenv' usada no codigo mas ausente do package.json (adicionada); e o arquivo db/schema.sql nao foi extraido automaticamente (cabecalho com nome de arquivo entre parenteses no meio da frase, fora do padrao de extracao - criado manualmente com o conteudo exato do .md original, e o extrator foi atualizado para esse padrao). Seguranca: bcrypt correto, autenticacao via Bearer token (token nao enviado automaticamente pelo navegador em requisicoes cross-site, logo sem exposicao a CSRF por arquitetura), sem admin padrao (autocadastro publico). Segredo JWT com fallback rotulado (nao hardcoded puro).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arquitetura diferente da tentativa 1: usa cookie de sessao em vez de Bearer token. bcrypt correto (confirmado no banco), bloqueio sem token funcional. Porem cookie SEM atributo SameSite (confirmado via header Set-Cookie bruto) - mesma lacuna de CSRF real encontrada no Gemini nivel 4. Segredo JWT hardcoded com fallback ('supersecretkey'). Inconsistencia arquitetural relevante entre as duas tentativas do mesmo modelo neste nivel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interativo (readline) e via argumento; ambos testados com sucesso. CSV com cabecalho, escapamento RFC 4180 completo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gemini-3.1-pro-preview</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Via argumento de linha de comando. Testado: duas execucoes, CSV com 2 linhas e cabecalho, sem sobrescrever.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interativo e via argumento. Testado: duas execucoes, CSV com cabecalho, sem sobrescrever.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interativo e via argumento. Testado: duas execucoes, CSV sem cabecalho mas sem sobrescrever.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLI com parsing manual de argumentos (--name/--email/--dob). CRUD completo testado: cadastro, duplicidade de e-mail rejeitada, atualizacao, remocao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menu interativo via readline; testavel neste sandbox apenas com delay artificial entre respostas simuladas (limitacao de teste, nao do codigo). Cadastro e listagem confirmados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLI com aliases em portugues/ingles. CRUD completo testado, incluindo confirmacao de seguranca (--sim) exigida para remocao - boa pratica, nao bug.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 correcoes manuais: better-sqlite3^9.4.3 sem binario pre-compilado (subido para ^12.2.0); chalk^5.3.0 e ESM-only, incompativel com require() do codigo (rebaixado para ^4.1.2). Apos corrigir, CRUD completo funcional com duplicidade rejeitada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API REST completa testada via HTTP real: criar, listar, 409 em duplicidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API REST completa testada via HTTP real: criar, listar, 409 em duplicidade, prepared statements explicitos documentados no codigo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API REST completa testada via HTTP real: criar, listar, 409 em duplicidade, envelope {dados,total} consistente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 correcoes manuais: comentario invalido '// package.json' dentro do proprio JSON (extrator atualizado para remover automaticamente); codigo nao criava o diretorio data/ necessario para o SQLite (SQLITE_CANTOPEN ate criar manualmente). Apos corrigir, CRUD completo funcional.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend + API REST completos testados via HTTP real: criar, listar, 409 em duplicidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend + API REST funcionais, mas com duas ressalvas de qualidade: porta hardcoded em 3000 (ignora variavel de ambiente PORT) e erro bruto do SQLite (UNIQUE constraint) vazado diretamente na resposta ao cliente em vez de mensagem amigavel (400 em vez de 409).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend + API REST completos testados via HTTP real: criar, listar, 409 em duplicidade, mensagens em portugues consistentes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 correcao manual: dependencia 'cors' usada no codigo mas ausente do package.json (adicionada). Estrutura frontend/backend separada (nao e defeito, e escolha arquitetural valida). Apos corrigir, CRUD completo via HTTP real funcional.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autenticacao Bearer token completa testada: listagem publica, bloqueio sem token (401), registro, login, hash bcrypt confirmado no banco. Segredo JWT com fallback rotulado (nao hardcoded puro). ESLint reportou 12 avisos brutos, mas 11 sao falso-positivo de ambiente (localStorage/funcoes chamadas via onclick em public/app.js, arquivo de navegador lintado com regras de Node.js) - apenas 1 aviso real (variavel 'err' nao utilizada).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autenticacao por cookie completa testada: listagem publica, bloqueio sem token (401), login com credencial administrativa padrao fraca (admin/admin123) criada automaticamente e funcional de primeira - terceira ocorrencia identica nas tres tentativas deste nivel. Segredo JWT hardcoded sem fallback via variavel de ambiente. Cookie sem atributo SameSite.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autenticacao por sessao (cookie) com formularios server-side testada de ponta a ponta: bloqueio sem login (302 redirect), criacao de admin via script dedicado (sem credencial padrao), login funcional, sessao autenticada confirmada, hash scrypt binario no banco. Token de sessao criptografico (crypto.randomBytes), token CSRF dedicado, cookie SameSite=strict.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autenticacao Bearer token completa testada: listagem publica, bloqueio sem token (401), registro publico (sem admin padrao), login retornando JWT valido. Segredo JWT com fallback rotulado.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo agregado por provedor</t>
@@ -370,9 +472,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -543,7 +646,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -628,7 +731,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1027,7 +1146,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -2379,6 +2498,1234 @@
         <v>105</v>
       </c>
     </row>
+    <row r="33" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E33" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="21" t="n">
+        <v>6030</v>
+      </c>
+      <c r="G33" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H33" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J33" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L33" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M33" s="22" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D34" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E34" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="21" t="n">
+        <v>5531</v>
+      </c>
+      <c r="G34" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H34" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J34" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L34" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M34" s="22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D35" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E35" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="21" t="n">
+        <v>13346</v>
+      </c>
+      <c r="G35" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H35" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J35" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L35" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M35" s="22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C36" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D36" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E36" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" s="21" t="n">
+        <v>13965</v>
+      </c>
+      <c r="G36" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H36" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I36" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J36" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L36" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M36" s="22" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E37" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="21" t="n">
+        <v>11994</v>
+      </c>
+      <c r="G37" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H37" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J37" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L37" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M37" s="22" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D38" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E38" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" s="21" t="n">
+        <v>11651</v>
+      </c>
+      <c r="G38" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H38" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J38" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L38" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M38" s="22" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B39" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D39" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E39" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="21" t="n">
+        <v>14221</v>
+      </c>
+      <c r="G39" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H39" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J39" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L39" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M39" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E40" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" s="21" t="n">
+        <v>14567</v>
+      </c>
+      <c r="G40" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H40" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J40" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L40" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M40" s="22" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="202.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B41" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C41" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D41" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E41" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="21" t="n">
+        <v>11772</v>
+      </c>
+      <c r="G41" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H41" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J41" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="M41" s="22" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B42" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E42" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" s="21" t="n">
+        <v>14388</v>
+      </c>
+      <c r="G42" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H42" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J42" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="L42" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="M42" s="22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B43" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D43" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E43" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="21" t="n">
+        <v>16348</v>
+      </c>
+      <c r="G43" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H43" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J43" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L43" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M43" s="22" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B44" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D44" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E44" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" s="21" t="n">
+        <v>3421</v>
+      </c>
+      <c r="G44" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H44" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J44" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L44" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M44" s="22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B45" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D45" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E45" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" s="21" t="n">
+        <v>3843</v>
+      </c>
+      <c r="G45" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H45" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J45" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L45" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M45" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B46" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D46" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E46" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="21" t="n">
+        <v>6146</v>
+      </c>
+      <c r="G46" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H46" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J46" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L46" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M46" s="22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E47" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="21" t="n">
+        <v>16263</v>
+      </c>
+      <c r="G47" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H47" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J47" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L47" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M47" s="22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E48" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="21" t="n">
+        <v>8189</v>
+      </c>
+      <c r="G48" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H48" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J48" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L48" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M48" s="22" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D49" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E49" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="21" t="n">
+        <v>23557</v>
+      </c>
+      <c r="G49" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H49" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J49" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L49" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M49" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C50" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D50" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E50" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" s="21" t="n">
+        <v>13266</v>
+      </c>
+      <c r="G50" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H50" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I50" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J50" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L50" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M50" s="22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C51" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D51" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E51" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F51" s="21" t="n">
+        <v>19857</v>
+      </c>
+      <c r="G51" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H51" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J51" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L51" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M51" s="22" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C52" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D52" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E52" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="21" t="n">
+        <v>6999</v>
+      </c>
+      <c r="G52" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H52" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J52" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L52" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M52" s="22" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C53" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D53" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E53" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" s="21" t="n">
+        <v>15580</v>
+      </c>
+      <c r="G53" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H53" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J53" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L53" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M53" s="22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C54" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D54" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E54" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" s="21" t="n">
+        <v>12082</v>
+      </c>
+      <c r="G54" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H54" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="I54" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J54" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L54" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M54" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B55" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C55" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D55" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E55" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" s="21" t="n">
+        <v>18873</v>
+      </c>
+      <c r="G55" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H55" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J55" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L55" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M55" s="22" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B56" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C56" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D56" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E56" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" s="21" t="n">
+        <v>10857</v>
+      </c>
+      <c r="G56" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H56" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J56" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="K56" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L56" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M56" s="22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B57" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C57" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D57" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E57" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F57" s="21" t="n">
+        <v>36307</v>
+      </c>
+      <c r="G57" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H57" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J57" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L57" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M57" s="22" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B58" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C58" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D58" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E58" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F58" s="21" t="n">
+        <v>15766</v>
+      </c>
+      <c r="G58" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H58" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J58" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L58" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="M58" s="22" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B59" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C59" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D59" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E59" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F59" s="21" t="n">
+        <v>18384</v>
+      </c>
+      <c r="G59" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H59" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J59" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L59" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="M59" s="22" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B60" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C60" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D60" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E60" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F60" s="21" t="n">
+        <v>14231</v>
+      </c>
+      <c r="G60" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H60" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J60" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="K60" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="L60" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="M60" s="22" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B61" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C61" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D61" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E61" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>45058</v>
+      </c>
+      <c r="G61" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H61" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J61" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="K61" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L61" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="M61" s="22" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B62" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C62" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D62" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E62" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F62" s="21" t="n">
+        <v>17001</v>
+      </c>
+      <c r="G62" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="H62" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J62" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L62" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="M62" s="22" t="s">
+        <v>139</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
@@ -2398,7 +3745,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -2412,7 +3759,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>106</v>
+        <v>140</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2423,7 +3770,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>107</v>
+        <v>141</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2437,50 +3784,50 @@
         <v>28</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>108</v>
+        <v>142</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>109</v>
+        <v>143</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>110</v>
+        <v>144</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>111</v>
+        <v>145</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>112</v>
+        <v>146</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>113</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="21" t="n">
-        <f aca="false">IFERROR(COUNTIFS(Avaliacao!C3:C32,A5,Avaliacao!G3:G32,"S")/COUNTIFS(Avaliacao!C3:C32,A5,Avaliacao!G3:G32,"&lt;&gt;")*100,"")</f>
+      <c r="B5" s="23" t="n">
+        <f aca="false">IFERROR(COUNTIFS(Avaliacao!C3:C62,A5,Avaliacao!G3:G62,"S")/COUNTIFS(Avaliacao!C3:C62,A5,Avaliacao!G3:G62,"&lt;&gt;")*100,"")</f>
         <v>100</v>
       </c>
-      <c r="C5" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!H3:H32,Avaliacao!C3:C32,A5),"")</f>
-        <v>0</v>
-      </c>
-      <c r="D5" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!I3:I32,Avaliacao!C3:C32,A5),"")</f>
-        <v>4.8</v>
-      </c>
-      <c r="E5" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!J3:J32,Avaliacao!C3:C32,A5),"")</f>
-        <v>1.5</v>
-      </c>
-      <c r="F5" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!K3:K32,Avaliacao!C3:C32,A5),"")</f>
-        <v>4.8</v>
-      </c>
-      <c r="G5" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!L3:L32,Avaliacao!C3:C32,A5,Avaliacao!A3:A32,4),"")</f>
+      <c r="C5" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!H3:H62,Avaliacao!C3:C62,A5),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!I3:I62,Avaliacao!C3:C62,A5),"")</f>
+        <v>4.86666666666667</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!J3:J62,Avaliacao!C3:C62,A5),"")</f>
+        <v>1.2</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!K3:K62,Avaliacao!C3:C62,A5),"")</f>
+        <v>4.86666666666667</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!L3:L62,Avaliacao!C3:C62,A5,Avaliacao!A3:A62,4),"")</f>
         <v>4</v>
       </c>
     </row>
@@ -2488,28 +3835,28 @@
       <c r="A6" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="21" t="n">
-        <f aca="false">IFERROR(COUNTIFS(Avaliacao!C3:C32,A6,Avaliacao!G3:G32,"S")/COUNTIFS(Avaliacao!C3:C32,A6,Avaliacao!G3:G32,"&lt;&gt;")*100,"")</f>
+      <c r="B6" s="23" t="n">
+        <f aca="false">IFERROR(COUNTIFS(Avaliacao!C3:C62,A6,Avaliacao!G3:G62,"S")/COUNTIFS(Avaliacao!C3:C62,A6,Avaliacao!G3:G62,"&lt;&gt;")*100,"")</f>
         <v>100</v>
       </c>
-      <c r="C6" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!H3:H32,Avaliacao!C3:C32,A6),"")</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!I3:I32,Avaliacao!C3:C32,A6),"")</f>
-        <v>5</v>
-      </c>
-      <c r="E6" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!J3:J32,Avaliacao!C3:C32,A6),"")</f>
-        <v>0.7</v>
-      </c>
-      <c r="F6" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!K3:K32,Avaliacao!C3:C32,A6),"")</f>
-        <v>4.9</v>
-      </c>
-      <c r="G6" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!L3:L32,Avaliacao!C3:C32,A6,Avaliacao!A3:A32,4),"")</f>
+      <c r="C6" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!H3:H62,Avaliacao!C3:C62,A6),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!I3:I62,Avaliacao!C3:C62,A6),"")</f>
+        <v>5</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!J3:J62,Avaliacao!C3:C62,A6),"")</f>
+        <v>0.866666666666667</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!K3:K62,Avaliacao!C3:C62,A6),"")</f>
+        <v>4.93333333333333</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!L3:L62,Avaliacao!C3:C62,A6,Avaliacao!A3:A62,4),"")</f>
         <v>5</v>
       </c>
     </row>
@@ -2517,29 +3864,58 @@
       <c r="A7" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="21" t="n">
-        <f aca="false">IFERROR(COUNTIFS(Avaliacao!C3:C32,A7,Avaliacao!G3:G32,"S")/COUNTIFS(Avaliacao!C3:C32,A7,Avaliacao!G3:G32,"&lt;&gt;")*100,"")</f>
+      <c r="B7" s="23" t="n">
+        <f aca="false">IFERROR(COUNTIFS(Avaliacao!C3:C62,A7,Avaliacao!G3:G62,"S")/COUNTIFS(Avaliacao!C3:C62,A7,Avaliacao!G3:G62,"&lt;&gt;")*100,"")</f>
         <v>100</v>
       </c>
-      <c r="C7" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!H3:H32,Avaliacao!C3:C32,A7),"")</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!I3:I32,Avaliacao!C3:C32,A7),"")</f>
-        <v>4.4</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!J3:J32,Avaliacao!C3:C32,A7),"")</f>
-        <v>0.7</v>
-      </c>
-      <c r="F7" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!K3:K32,Avaliacao!C3:C32,A7),"")</f>
-        <v>3.4</v>
-      </c>
-      <c r="G7" s="21" t="n">
-        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!L3:L32,Avaliacao!C3:C32,A7,Avaliacao!A3:A32,4),"")</f>
-        <v>3</v>
+      <c r="C7" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!H3:H62,Avaliacao!C3:C62,A7),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!I3:I62,Avaliacao!C3:C62,A7),"")</f>
+        <v>4.6</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!J3:J62,Avaliacao!C3:C62,A7),"")</f>
+        <v>0.733333333333333</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!K3:K62,Avaliacao!C3:C62,A7),"")</f>
+        <v>3.6</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!L3:L62,Avaliacao!C3:C62,A7,Avaliacao!A3:A62,4),"")</f>
+        <v>2.66666666666667</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8" s="25" t="n">
+        <f aca="false">IFERROR(COUNTIFS(Avaliacao!C3:C62,A8,Avaliacao!G3:G62,"S")/COUNTIFS(Avaliacao!C3:C62,A8,Avaliacao!G3:G62,"&lt;&gt;")*100,"")</f>
+        <v>100</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!H3:H62,Avaliacao!C3:C62,A8),"")</f>
+        <v>0.733333333333333</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!I3:I62,Avaliacao!C3:C62,A8),"")</f>
+        <v>5</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!J3:J62,Avaliacao!C3:C62,A8),"")</f>
+        <v>0.533333333333333</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!K3:K62,Avaliacao!C3:C62,A8),"")</f>
+        <v>4.35714285714286</v>
+      </c>
+      <c r="G8" s="25" t="n">
+        <f aca="false">IFERROR(AVERAGEIFS(Avaliacao!L3:L62,Avaliacao!C3:C62,A8,Avaliacao!A3:A62,4),"")</f>
+        <v>3.66666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>